<commit_message>
Update 6 files\n\nCo-authored-by: Freebuff Agent <agent@mail.freebuff.app>
</commit_message>
<xml_diff>
--- a/Nicky_Clean_Input.xlsx
+++ b/Nicky_Clean_Input.xlsx
@@ -2017,7 +2017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2035,7 +2035,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SHEETS</t>
+          <t>DELIVERABLES</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -2043,36 +2043,36 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ties</t>
+          <t>Nicky_Relative_Input.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>One row per station in survey order. DeltaG(row i) = g(i) - g(i-1).</t>
+          <t>RELATIVE observations: Station + DeltaG (tie into each station).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Base Reference</t>
+          <t>Nicky_Absolute_Input.xlsx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Absolute anchors for the network (START + 5 GCP/GTS controls).</t>
+          <t>ABSOLUTE values: Station + KnownG + Sigma (base/control anchors).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Nicky_Clean_Input.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>This sheet.</t>
+          <t>Both above + documentation, in one workbook.</t>
         </is>
       </c>
     </row>
@@ -2083,7 +2083,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TIES - COLUMN GUIDE</t>
+          <t>RELATIVE FILE - COLUMN GUIDE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -2211,7 +2211,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ANCHORS</t>
+          <t>ABSOLUTE FILE - ANCHORS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -2263,126 +2263,122 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>STATION 2</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Occupied but no DeltaG recorded in the sheet; kept as the 'from' station of tie 2-&gt;1.</t>
-        </is>
-      </c>
+          <t>NETWORK SUMMARY (validated)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Rows</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>96 (incl. START anchor + closing leg back to START).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NETWORK SUMMARY (validated)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+          <t>Loop misclosure</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>7.581 uGal (distributed as residuals by the adjustment).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rows</t>
+          <t>Rank / dof</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>96 (incl. START anchor + closing leg back to START).</t>
+          <t>Full rank; obs=100, unknowns=94, dof=6 (partial mode).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Loop misclosure</t>
+          <t>vs sheet's official values</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>7.581 uGal (distributed as residuals by the adjustment).</t>
+          <t>52 stations compared, RMS 0.001 uGal, max 0.001 uGal (partial mode);</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Rank / dof</t>
-        </is>
-      </c>
+      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Full rank; obs=100, unknowns=94, dof=6 (partial mode).</t>
+          <t>47 stations, RMS 0.000 uGal (hard-fixed mode).</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>vs sheet's official values</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>52 stations compared, RMS 0.001 uGal, max 0.001 uGal (partial mode);</t>
-        </is>
-      </c>
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>47 stations, RMS 0.000 uGal (hard-fixed mode).</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>HOW TO USE</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>In the app, run 'Least Squares Adjustment'.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HOW TO USE</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Load Nicky_Relative_Input.xlsx as the day/survey file and</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>In the app, run 'Least Squares Adjustment'.</t>
+          <t>Nicky_Absolute_Input.xlsx as the base station reference file.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
-        <is>
-          <t>Load 'Ties' as the day/survey file and 'Base Reference' as the base station file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
         <is>
           <t>Pick a weighting scheme and run - results match the survey sheet's final values.</t>
         </is>

</xml_diff>